<commit_message>
Matrice mise à jour automatiquement (20/10/2026 18:27)
</commit_message>
<xml_diff>
--- a/matrices/MATRICE_DE_SUIVI_DES_ACTIVITES_du_20-10-26.xlsx
+++ b/matrices/MATRICE_DE_SUIVI_DES_ACTIVITES_du_20-10-26.xlsx
@@ -17,8 +17,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -220,7 +220,7 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -398,7 +398,7 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -407,7 +407,12 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -965,7 +970,7 @@
       </c>
       <c r="P4" s="28" t="n"/>
       <c r="Q4" s="28" t="n"/>
-      <c r="R4" s="67" t="n">
+      <c r="R4" s="73" t="n">
         <v>46315</v>
       </c>
       <c r="S4" s="11" t="inlineStr">
@@ -1106,13 +1111,15 @@
           <t>24/08/2026 - 24/12/2026</t>
         </is>
       </c>
-      <c r="K6" s="23" t="n"/>
+      <c r="K6" s="74" t="n">
+        <v>46315</v>
+      </c>
       <c r="L6" s="26" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="M6" s="27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demarrage effectif </t>
+          <t>Travaux en cours</t>
         </is>
       </c>
       <c r="N6" s="22" t="inlineStr">
@@ -1122,7 +1129,7 @@
       </c>
       <c r="O6" s="22" t="inlineStr">
         <is>
-          <t>AGIR pour ODD</t>
+          <t>ONG EPC</t>
         </is>
       </c>
       <c r="P6" s="28" t="n"/>
@@ -2771,7 +2778,7 @@
       <c r="J30" s="49" t="n"/>
       <c r="K30" s="49" t="n"/>
       <c r="L30" s="52" t="n">
-        <v>8.65</v>
+        <v>8.85</v>
       </c>
       <c r="M30" s="48" t="n"/>
       <c r="N30" s="50" t="n"/>
@@ -3422,7 +3429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3505,7 +3512,7 @@
       <c r="A2" t="n">
         <v>897535549</v>
       </c>
-      <c r="B2" s="72" t="n">
+      <c r="B2" s="75" t="n">
         <v>46315</v>
       </c>
       <c r="C2" t="n">
@@ -3552,6 +3559,60 @@
       <c r="L2" t="inlineStr">
         <is>
           <t>2026-10-20 17:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>897563476</v>
+      </c>
+      <c r="B3" s="75" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>BAGOUE</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>BOUNDIALI</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>SELECT IVOIREMULTISERVICES SARL</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Travaux en cours</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>10</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>ONG EPC</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>superviseur</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-10-20 18:26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Matrice mise à jour automatiquement (20/10/2026 18:39)
</commit_message>
<xml_diff>
--- a/matrices/MATRICE_DE_SUIVI_DES_ACTIVITES_du_20-10-26.xlsx
+++ b/matrices/MATRICE_DE_SUIVI_DES_ACTIVITES_du_20-10-26.xlsx
@@ -16,8 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -219,7 +220,7 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -412,6 +413,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -948,26 +950,30 @@
           <t>17/08/2026 - 17/12/2026</t>
         </is>
       </c>
-      <c r="K4" s="23" t="n"/>
+      <c r="K4" s="74" t="n">
+        <v>46315</v>
+      </c>
       <c r="L4" s="26" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="M4" s="27" t="inlineStr">
         <is>
-          <t>Travaux en cours</t>
+          <t>Travaux achevés</t>
         </is>
       </c>
       <c r="N4" s="22" t="inlineStr">
         <is>
-          <t>Pas de PGES</t>
+          <t>Validé</t>
         </is>
       </c>
       <c r="O4" s="22" t="inlineStr">
         <is>
-          <t>ONG EPC</t>
-        </is>
-      </c>
-      <c r="P4" s="28" t="n"/>
+          <t>KERA-SY-IRÊ</t>
+        </is>
+      </c>
+      <c r="P4" s="76" t="n">
+        <v>46315</v>
+      </c>
       <c r="Q4" s="28" t="n"/>
       <c r="R4" s="73" t="n">
         <v>46315</v>
@@ -2777,7 +2783,7 @@
       <c r="J30" s="49" t="n"/>
       <c r="K30" s="49" t="n"/>
       <c r="L30" s="52" t="n">
-        <v>8.85</v>
+        <v>10.77</v>
       </c>
       <c r="M30" s="48" t="n"/>
       <c r="N30" s="50" t="n"/>
@@ -3428,7 +3434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3615,6 +3621,60 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>897569755</v>
+      </c>
+      <c r="B4" s="75" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>BAFING</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>KORO</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>NATHA SARL</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Travaux achevés</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>100</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>KERA-SY-IRÊ</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>gar_principal</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-10-20 18:39</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>